<commit_message>
auto: 작업 자동 저장 2026-07-24 09:44
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval-runner/orchestrator/data/RC2/06_calibration/RC2_judge_캘리브레이션_판정30_v1_0.xlsx
+++ b/eval-runner/orchestrator/data/RC2/06_calibration/RC2_judge_캘리브레이션_판정30_v1_0.xlsx
@@ -492,7 +492,6 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -521,8 +520,6 @@
           <t>'설치 불필요(무설치)'와 '웹 브라우저만으로 접속' 두 요소를 모두 포함하면 정답</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -551,8 +548,6 @@
           <t>정답에 필수 요소(파일 전송 사용여부 선택)가 포함되면 pass.</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -581,8 +576,6 @@
           <t>'보안 솔루션 구축'을 포함하고 출처 unit_id가 일치</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -611,8 +604,6 @@
           <t>금융·공공 분야 공략과 글로벌 시장 우위 유지 언급이 모두 포함</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -641,8 +632,6 @@
           <t>'상담도구관리' 명칭을 언급</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -671,8 +660,6 @@
           <t>정답에 '6인 이하'와 '화상 회의 장비'가 모두 포함</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -701,8 +688,6 @@
           <t>허용 문자 조합과 50자 이하 제약을 언급</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -731,8 +716,6 @@
           <t>정답에 'AV Switcher', 'Audio Mixer', 'Amp'가 모두 포함</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -761,8 +744,6 @@
           <t>정답에 필수 요소(E-mail 주소 아는 경우, email 전송 기능)가 모두 포함되면 pass.</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -791,8 +772,6 @@
           <t>관리자 페이지 &gt; 상담 도구 관리 &gt; 상담 구분 경로를 언급</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -821,8 +800,6 @@
           <t>정답에 '판서', 'QR 코드', '공유'가 모두 포함</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -851,8 +828,6 @@
           <t>멀티 세션 지원과 3/5 session 규모를 언급</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -881,8 +856,6 @@
           <t>코퍼스에 근거가 없음을 밝히고 답변을 거부/보류하면 정답 (임의 금액 제시는 오답)</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -911,8 +884,6 @@
           <t>정답에 필수 요소(로그인 실패 5회, 설정 시간만큼 제한)가 모두 포함되면 pass.</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -941,8 +912,6 @@
           <t>정답에 필수 요소(아이디 수정 불가)가 포함되면 pass.</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -971,8 +940,6 @@
           <t>'190,000원'을 정확히 포함해야 정답</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1001,8 +968,6 @@
           <t>사전 예고 없는 변경 가능 취지 포함, 근거 출처 일치</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1031,8 +996,6 @@
           <t>사전 서면 동의 필요와 저작권법 저촉 포함, 근거 출처 일치</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1061,8 +1024,6 @@
           <t>고객이 언제든 화면 전송 중단 가능 취지 포함, 근거 출처 일치</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1091,8 +1052,6 @@
           <t>오디오 효과 설정 가능 취지 포함, 근거 출처 일치</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1121,8 +1080,6 @@
           <t>대기 화면이 지원 화면으로 전환됨을 명시</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1151,8 +1108,6 @@
           <t>공유화면 중 일부를 상담사가 못 보도록 차단한다는 기능을 설명하면 합격</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1181,8 +1136,6 @@
           <t>'일괄 에이전트 삭제' 명칭 포함, 근거 출처 일치</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1211,8 +1164,6 @@
           <t>필수 요소(안드로이드, 원격 제어)를 모두 포함하고 출처 unit_id가 RC2-HTTPSW-1299와 일치</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1241,8 +1192,6 @@
           <t>화면공유 사용 상태 조건과 캡쳐 가능 포함, 근거 출처 일치</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1271,8 +1220,6 @@
           <t>필수 요소(전 세계, 원격 연결) 모두 포함 + 근거 출처 일치</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1301,8 +1248,6 @@
           <t>필수 요소(컴퓨터 사용, 원격 지원) 모두 포함 + 근거 출처 일치</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1331,8 +1276,6 @@
           <t>'상담일지', '옵션', '적용' 요소가 모두 포함되면 합격</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1361,8 +1304,6 @@
           <t>'url'과 'SMS 링크' 두 요소를 모두 포함해야 정답</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
auto: 작업 자동 저장 2026-07-24 09:49
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval-runner/orchestrator/data/RC2/06_calibration/RC2_judge_캘리브레이션_판정30_v1_0.xlsx
+++ b/eval-runner/orchestrator/data/RC2/06_calibration/RC2_judge_캘리브레이션_판정30_v1_0.xlsx
@@ -491,7 +491,11 @@
           <t>정답에 'RSUPPORT SMARTBOARD'가 포함</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">

</xml_diff>

<commit_message>
auto: 작업 자동 저장 2026-07-24 09:55
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval-runner/orchestrator/data/RC2/06_calibration/RC2_judge_캘리브레이션_판정30_v1_0.xlsx
+++ b/eval-runner/orchestrator/data/RC2/06_calibration/RC2_judge_캘리브레이션_판정30_v1_0.xlsx
@@ -524,6 +524,11 @@
           <t>'설치 불필요(무설치)'와 '웹 브라우저만으로 접속' 두 요소를 모두 포함하면 정답</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -552,6 +557,11 @@
           <t>정답에 필수 요소(파일 전송 사용여부 선택)가 포함되면 pass.</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -580,6 +590,11 @@
           <t>'보안 솔루션 구축'을 포함하고 출처 unit_id가 일치</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>불합격</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -608,6 +623,11 @@
           <t>금융·공공 분야 공략과 글로벌 시장 우위 유지 언급이 모두 포함</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -636,6 +656,11 @@
           <t>'상담도구관리' 명칭을 언급</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -664,6 +689,11 @@
           <t>정답에 '6인 이하'와 '화상 회의 장비'가 모두 포함</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -692,6 +722,11 @@
           <t>허용 문자 조합과 50자 이하 제약을 언급</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -720,6 +755,11 @@
           <t>정답에 'AV Switcher', 'Audio Mixer', 'Amp'가 모두 포함</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -748,6 +788,11 @@
           <t>정답에 필수 요소(E-mail 주소 아는 경우, email 전송 기능)가 모두 포함되면 pass.</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -776,6 +821,11 @@
           <t>관리자 페이지 &gt; 상담 도구 관리 &gt; 상담 구분 경로를 언급</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -804,6 +854,11 @@
           <t>정답에 '판서', 'QR 코드', '공유'가 모두 포함</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -832,6 +887,11 @@
           <t>멀티 세션 지원과 3/5 session 규모를 언급</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -860,6 +920,11 @@
           <t>코퍼스에 근거가 없음을 밝히고 답변을 거부/보류하면 정답 (임의 금액 제시는 오답)</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>불합격</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -888,6 +953,11 @@
           <t>정답에 필수 요소(로그인 실패 5회, 설정 시간만큼 제한)가 모두 포함되면 pass.</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -916,6 +986,11 @@
           <t>정답에 필수 요소(아이디 수정 불가)가 포함되면 pass.</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -944,6 +1019,11 @@
           <t>'190,000원'을 정확히 포함해야 정답</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -972,6 +1052,11 @@
           <t>사전 예고 없는 변경 가능 취지 포함, 근거 출처 일치</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1000,6 +1085,11 @@
           <t>사전 서면 동의 필요와 저작권법 저촉 포함, 근거 출처 일치</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1028,6 +1118,11 @@
           <t>고객이 언제든 화면 전송 중단 가능 취지 포함, 근거 출처 일치</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1056,6 +1151,11 @@
           <t>오디오 효과 설정 가능 취지 포함, 근거 출처 일치</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1084,6 +1184,11 @@
           <t>대기 화면이 지원 화면으로 전환됨을 명시</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1112,6 +1217,11 @@
           <t>공유화면 중 일부를 상담사가 못 보도록 차단한다는 기능을 설명하면 합격</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1140,6 +1250,11 @@
           <t>'일괄 에이전트 삭제' 명칭 포함, 근거 출처 일치</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1168,6 +1283,11 @@
           <t>필수 요소(안드로이드, 원격 제어)를 모두 포함하고 출처 unit_id가 RC2-HTTPSW-1299와 일치</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1196,6 +1316,11 @@
           <t>화면공유 사용 상태 조건과 캡쳐 가능 포함, 근거 출처 일치</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1224,6 +1349,11 @@
           <t>필수 요소(전 세계, 원격 연결) 모두 포함 + 근거 출처 일치</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>불합격</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1252,6 +1382,11 @@
           <t>필수 요소(컴퓨터 사용, 원격 지원) 모두 포함 + 근거 출처 일치</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>불합격</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1278,6 +1413,11 @@
       <c r="E30" t="inlineStr">
         <is>
           <t>'상담일지', '옵션', '적용' 요소가 모두 포함되면 합격</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>합격</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 작업 자동 저장 2026-07-24 10:05
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval-runner/orchestrator/data/RC2/06_calibration/RC2_judge_캘리브레이션_판정30_v1_0.xlsx
+++ b/eval-runner/orchestrator/data/RC2/06_calibration/RC2_judge_캘리브레이션_판정30_v1_0.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>불합격</t>
+          <t>합격</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>불합격</t>
+          <t>합격</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>불합격</t>
+          <t>합격</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 작업 자동 저장 2026-07-24 10:06
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval-runner/orchestrator/data/RC2/06_calibration/RC2_judge_캘리브레이션_판정30_v1_0.xlsx
+++ b/eval-runner/orchestrator/data/RC2/06_calibration/RC2_judge_캘리브레이션_판정30_v1_0.xlsx
@@ -1384,7 +1384,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>불합격</t>
+          <t>합격</t>
         </is>
       </c>
     </row>
@@ -1446,6 +1446,11 @@
       <c r="E31" t="inlineStr">
         <is>
           <t>'url'과 'SMS 링크' 두 요소를 모두 포함해야 정답</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>합격</t>
         </is>
       </c>
     </row>

</xml_diff>